<commit_message>
El informe de migración habla en primera persona y nombra cada forma entera
La migración la hace una persona, y el informe y el Excel se lo dicen así a
quien anotó: «te pido», «he rellenado yo», «pregúntamelo». Lo que el editor
hará después no es corregir sino comprobar que la migración no dejó ningún
hueco. Ninguna arquitectura se nombra ya sin su forma —«una redondilla
octosílaba», «un soneto endecasílabo consonante»—, porque sola no dice nada;
el artículo se lee del nombre de la forma. La pestaña de instrucciones del
Excel dice «donde estás ahora» donde el informe dice «con este mismo texto».

El generador tolera un Excel abierto en Excel, que Windows bloquea: avisa,
salta ese fichero y sigue con los demás. Los ficheros de bloqueo «~$*.xlsx»
quedan fuera del repositorio.
</commit_message>
<xml_diff>
--- a/docs/dominio-metrico/migracion/cuestionarios/cegar-para-ver-mejor.xlsx
+++ b/docs/dominio-metrico/migracion/cuestionarios/cegar-para-ver-mejor.xlsx
@@ -21,25 +21,25 @@
     <t>Migración métrica · Cegar para ver mejor</t>
   </si>
   <si>
-    <t>Para Gabriel López · generado el 2026-09-19</t>
-  </si>
-  <si>
-    <t>El Excel tiene cinco pestañas. En tres de ellas hay que escribir —Responder, Confirmar y Desviaciones— y las otras dos son de consulta: Secuencias, con todo lo que tiene anotado tu obra, e Instrucciones, con este mismo texto. Solo hace falta escribir en las columnas de fondo amarillo, que son «Respuesta», «Excepciones / detalle» y «Comentario». El resto de columnas las genera el programa y las necesita tal cual para poder leer las respuestas, así que conviene no tocarlas.</t>
-  </si>
-  <si>
-    <t>En Responder están las preguntas que no hemos podido contestar con lo que ya tenías anotado. Cada fila corresponde a un pasaje y a una pregunta. Cuando la celda tiene desplegable, basta con elegir; cuando no, la columna «Cómo contestar» explica el formato. Las preguntas que se refieren a cada estrofa aparecen de dos maneras: si son pocas estrofas, hay una fila por estrofa; si son muchas, hay una sola fila cuya respuesta vale para todas, y las estrofas que se aparten de ella se anotan en «Excepciones / detalle» indicando los versos y la respuesta, por ejemplo «191–194: Cruzada · abab; 203–206: Cruzada · abab».</t>
-  </si>
-  <si>
-    <t>Las filas marcadas como Decidir señalan pasajes cuyo número de versos no encaja con la forma que tienen asignada. En ellas hay que elegir en el desplegable qué ocurre y explicarlo al lado. Si se trata de una laguna que no se contó, indica en qué verso está y cuántos versos faltan, porque los añadiremos a la numeración y todo lo que viene después se desplazará. Si lo que falla es el rango, escribe el rango correcto.</t>
-  </si>
-  <si>
-    <t>En Confirmar aparecen las respuestas que hemos rellenado nosotros a partir del término que elegiste en su día: la asonancia de un romance, el esquema de una octava real «regular», o que un endecasílabo suelto «puro» no lleva pareados. Solo hay que revisarlas. Si alguna no es así, elige «No es así» y escribe al lado lo que corresponde.</t>
+    <t>Para Gabriel López · generado el 2026-09-20</t>
+  </si>
+  <si>
+    <t>El Excel tiene cinco pestañas. En tres de ellas hay que escribir —Responder, Confirmar y Desviaciones— y las otras dos son de consulta: Secuencias, con todo lo que tiene anotado tu obra, e Instrucciones, donde estás ahora. Solo hace falta escribir en las columnas de fondo amarillo, que son «Respuesta», «Excepciones / detalle» y «Comentario». El resto de columnas las genera el programa y las necesita tal cual para poder leer las respuestas, así que conviene no tocarlas.</t>
+  </si>
+  <si>
+    <t>En Responder están las preguntas que no he podido contestar con lo que ya tenías anotado. Cada fila corresponde a un pasaje y a una pregunta. Cuando la celda tiene desplegable, basta con elegir; cuando no, la columna «Cómo contestar» explica el formato. Las preguntas que se refieren a cada estrofa aparecen de dos maneras: si son pocas estrofas, hay una fila por estrofa; si son muchas, hay una sola fila cuya respuesta vale para todas, y las estrofas que se aparten de ella se anotan en «Excepciones / detalle» indicando los versos y la respuesta, por ejemplo «191–194: Cruzada · abab; 203–206: Cruzada · abab».</t>
+  </si>
+  <si>
+    <t>Las filas marcadas como Decidir señalan pasajes cuyo número de versos no encaja con la forma que tienen asignada. En ellas hay que elegir en el desplegable qué ocurre y explicarlo al lado. Si se trata de una laguna que no se contó, indica en qué verso está y cuántos versos faltan, porque los añadiré a la numeración y todo lo que viene después se desplazará. Si lo que falla es el rango, escribe el rango correcto.</t>
+  </si>
+  <si>
+    <t>En Confirmar aparecen las respuestas que he rellenado yo a partir del término que elegiste en su día: la asonancia de un romance, el esquema de una octava real «regular», o que un endecasílabo suelto «puro» no lleva pareados. Solo hay que revisarlas. Si alguna no es así, elige «No es así» y escribe al lado lo que corresponde.</t>
   </si>
   <si>
     <t>En Desviaciones están los versos hipométricos e hipermétricos, las rimas defectuosas y las lagunas que anotaste, con tus notas, y cómo quedan en el modelo nuevo. Se trasladan tal cual. Si tienes a mano el número de sílabas de algún verso hipométrico o hipermétrico, ponlo en la columna «Sílabas»; si no, se registra simplemente que el verso tiene menos o más sílabas de las que le tocan, sin dar una cifra.</t>
   </si>
   <si>
-    <t>Si algo no está claro o no sabes cómo contestarlo, pregúntaselo a David antes de dejarlo a medias. Una vez hecha la migración podrás ver cada secuencia de tu obra con el editor nuevo en el dashboard y corregir allí lo que haga falta.</t>
+    <t>Si algo no está claro o no sabes cómo contestarlo, pregúntamelo antes de dejarlo a medias. Una vez hecha la migración podrás ver cada secuencia de tu obra con el editor nuevo en el dashboard y comprobar allí que la migración no dejó ningún hueco.</t>
   </si>
   <si>
     <t>Cuando no hay desplegable, los formatos son estos:</t>

</xml_diff>

<commit_message>
Las instrucciones dejan de repetir lo que cada fila ya dice
La lista de formatos del final —medidas, posiciones, esquema de rima,
excepciones— repetía, con otras palabras, la columna «Cómo contestar» de las
filas que los usan: el mismo ejemplo de excepciones aparecía tres veces, y el
de la lista se explicaba a sí mismo diciendo «como arriba». Se va entera. Donde
hace falta saber un formato es en la fila que lo pide, y ahí sigue.

Con ella se va también el ejemplo del párrafo de Responder, que era el tercero,
y a cambio la fila que admite excepciones enseña dos, para que se vea que se
separan con punto y coma.
</commit_message>
<xml_diff>
--- a/docs/dominio-metrico/migracion/cuestionarios/cegar-para-ver-mejor.xlsx
+++ b/docs/dominio-metrico/migracion/cuestionarios/cegar-para-ver-mejor.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="63">
   <si>
     <t>Migración métrica · Cegar para ver mejor</t>
   </si>
@@ -27,7 +27,7 @@
     <t>El Excel tiene cinco pestañas. En tres de ellas hay que escribir —Responder, Confirmar y Desviaciones— y las otras dos son de consulta: Secuencias, con todo lo que tiene anotado tu obra, e Instrucciones, donde estás ahora. Solo hace falta escribir en las columnas de fondo amarillo, que son «Respuesta», «Excepciones / detalle» y «Comentario». El resto de columnas las genera el programa y las necesita tal cual para poder leer las respuestas, así que conviene no tocarlas.</t>
   </si>
   <si>
-    <t>En Responder están las preguntas que no he podido contestar con lo que ya tenías anotado. Cada fila corresponde a un pasaje y a una pregunta, también cuando la pregunta es de cada estrofa: se contesta una vez y la respuesta vale para todas, y las estrofas que se aparten se anotan en «Excepciones / detalle» como «versos: esquema», por ejemplo «191-194: abab; 203-206: abab». Cuando la celda tiene desplegable, basta con elegir; cuando no, la columna «Cómo contestar» explica el formato.</t>
+    <t>En Responder están las preguntas que no he podido contestar con lo que ya tenías anotado. Cada fila corresponde a un pasaje y a una pregunta, también cuando la pregunta es de cada estrofa: se contesta una vez y la respuesta vale para todas, y las estrofas que se aparten se anotan en «Excepciones / detalle». Cuando la celda tiene desplegable, basta con elegir; cuando no, la columna «Cómo contestar» dice el formato y da un ejemplo.</t>
   </si>
   <si>
     <t>Las filas marcadas como Decidir señalan pasajes cuyo número de versos no encaja con la forma que tienen asignada. En ellas hay que elegir en el desplegable qué ocurre y explicarlo al lado. Si se trata de una laguna que no se contó, indica en qué verso está y cuántos versos faltan, porque los añadiré a la numeración y todo lo que viene después se desplazará. Si lo que falla es el rango, escribe el rango correcto.</t>
@@ -40,21 +40,6 @@
   </si>
   <si>
     <t>Si algo no está claro o no sabes cómo contestarlo, pregúntamelo antes de dejarlo a medias. Una vez hecha la migración podrás ver cada secuencia de tu obra con el editor nuevo en el dashboard y comprobar allí que la migración no dejó ningún hueco.</t>
-  </si>
-  <si>
-    <t>Cuando no hay desplegable, los formatos son estos:</t>
-  </si>
-  <si>
-    <t>Medidas: el número de sílabas de cada verso, en orden y separados por espacios. Por ejemplo, «7 11 7 7 11 7 11 11».</t>
-  </si>
-  <si>
-    <t>Posiciones: en qué versos de la estrofa cae el quebrado y cuántas sílabas tiene cada uno, separados por comas. Por ejemplo, «3: 4, 8: 5» quiere decir que el verso 3 tiene cuatro sílabas y el 8 tiene cinco.</t>
-  </si>
-  <si>
-    <t>Esquema de rima: una letra por verso, en mayúscula si el verso es de arte mayor y un guion si queda suelto. Por ejemplo, «aBab-B».</t>
-  </si>
-  <si>
-    <t>Excepciones: los versos de la estrofa y su esquema, separados por dos puntos, y cada estrofa de la siguiente con punto y coma. Por ejemplo, «191-194: abab; 203-206: abab». El esquema se escribe como arriba: una letra por verso, en mayúscula si el verso es de arte mayor.</t>
   </si>
   <si>
     <t>lista</t>
@@ -284,14 +269,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -640,7 +624,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -684,31 +668,6 @@
     <row r="9" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -727,17 +686,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -762,36 +721,36 @@
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="G1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="H1" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="I1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="J1" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -817,120 +776,120 @@
     <col min="9" max="9" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H1" s="5" t="s">
+      <c r="F1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="I1" s="5" t="s">
-        <v>25</v>
+      <c r="H1" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="G2" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I2" s="6" t="s">
         <v>31</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="I2" s="7" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I3" s="6" t="s">
         <v>37</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="H3" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>45</v>
+        <v>29</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -962,36 +921,36 @@
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>25</v>
+    <row r="1" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1019,39 +978,39 @@
     <col min="11" max="11" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="I1" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1" s="5" t="s">
+      <c r="J1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1059,34 +1018,34 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="C2" s="3">
         <v>244</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1094,34 +1053,34 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C3" s="3">
         <v>176</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="G3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="J3" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="H3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>65</v>
-      </c>
       <c r="K3" s="3" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1129,34 +1088,34 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C4" s="3">
         <v>64</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>